<commit_message>
Simplify transaction upload template: remove phone and date columns, use upload timestamp
</commit_message>
<xml_diff>
--- a/public/templates/Transaction_Template.xlsx
+++ b/public/templates/Transaction_Template.xlsx
@@ -397,99 +397,79 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:F3"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="25.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="30.83203125" customWidth="1"/>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Phone</v>
+        <v>Customer Name</v>
       </c>
       <c r="B1" t="str">
-        <v>Customer Name</v>
+        <v>Type</v>
       </c>
       <c r="C1" t="str">
-        <v>Type</v>
+        <v>Quantity</v>
       </c>
       <c r="D1" t="str">
-        <v>Quantity</v>
+        <v>Vehicle No</v>
       </c>
       <c r="E1" t="str">
-        <v>Date</v>
+        <v>Deposit Amount</v>
       </c>
       <c r="F1" t="str">
-        <v>Vehicle No</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Deposit Amount</v>
-      </c>
-      <c r="H1" t="str">
         <v>Remarks</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>0771234567</v>
+        <v>Ruwan Agri Farm</v>
       </c>
       <c r="B2" t="str">
-        <v>Ruwan Agri Farm</v>
-      </c>
-      <c r="C2" t="str">
         <v>OUT</v>
       </c>
-      <c r="D2">
+      <c r="C2">
         <v>50</v>
       </c>
-      <c r="E2" t="str">
-        <v>2026-09-11 09:30</v>
+      <c r="D2" t="str">
+        <v>LK-3945</v>
+      </c>
+      <c r="E2">
+        <v>100000</v>
       </c>
       <c r="F2" t="str">
-        <v>LK-3945</v>
-      </c>
-      <c r="G2">
-        <v>100000</v>
-      </c>
-      <c r="H2" t="str">
         <v>Regular morning issue</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>0719876543</v>
+        <v>Kamal Stores</v>
       </c>
       <c r="B3" t="str">
-        <v>Kamal Stores</v>
-      </c>
-      <c r="C3" t="str">
         <v>IN</v>
       </c>
-      <c r="D3">
+      <c r="C3">
         <v>30</v>
       </c>
-      <c r="E3" t="str">
-        <v>2026-09-11 14:15</v>
+      <c r="D3" t="str">
+        <v>LN-4124</v>
+      </c>
+      <c r="E3">
+        <v>60000</v>
       </c>
       <c r="F3" t="str">
-        <v>LN-4124</v>
-      </c>
-      <c r="G3">
-        <v>60000</v>
-      </c>
-      <c r="H3" t="str">
         <v>Return from market</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>